<commit_message>
Created new branch UI_TESTING to experiment with how the chat interface will work
</commit_message>
<xml_diff>
--- a/Contact emails/CONTACT EMAILS.xlsx
+++ b/Contact emails/CONTACT EMAILS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Jonny/Desktop/University-chatbot/Contact emails/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3D3FBA4-6E96-4C41-847C-CE13CD3A5CB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8016D9A0-A11B-E548-B5EC-4F7D8C96B7C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="53">
   <si>
     <t>Department</t>
   </si>
@@ -109,9 +109,6 @@
     <t>Ipoint</t>
   </si>
   <si>
-    <t>IPoint Helpdesk</t>
-  </si>
-  <si>
     <t>Ipoint@huddersfield.com</t>
   </si>
   <si>
@@ -127,9 +124,6 @@
     <t>wellbeing@huddersfield.com</t>
   </si>
   <si>
-    <t>It Support</t>
-  </si>
-  <si>
     <t>IT support</t>
   </si>
   <si>
@@ -182,6 +176,9 @@
   </si>
   <si>
     <t>CristianoRonaldo@huddersfield.com</t>
+  </si>
+  <si>
+    <t>IT Support</t>
   </si>
 </sst>
 </file>
@@ -571,7 +568,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -582,7 +579,7 @@
         <v>5</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -593,7 +590,7 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -604,7 +601,7 @@
         <v>7</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -615,7 +612,7 @@
         <v>8</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -626,7 +623,7 @@
         <v>9</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
@@ -637,7 +634,7 @@
         <v>10</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
@@ -648,7 +645,7 @@
         <v>11</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
@@ -659,7 +656,7 @@
         <v>12</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
@@ -670,7 +667,7 @@
         <v>13</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -681,7 +678,7 @@
         <v>14</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
@@ -692,7 +689,7 @@
         <v>15</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
@@ -703,7 +700,7 @@
         <v>16</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
@@ -714,7 +711,7 @@
         <v>17</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
@@ -725,7 +722,7 @@
         <v>18</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
@@ -736,7 +733,7 @@
         <v>19</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
@@ -788,43 +785,43 @@
         <v>28</v>
       </c>
       <c r="B22" t="s">
+        <v>28</v>
+      </c>
+      <c r="C22" t="s">
         <v>29</v>
-      </c>
-      <c r="C22" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" t="s">
+        <v>30</v>
+      </c>
+      <c r="C23" t="s">
         <v>31</v>
-      </c>
-      <c r="B23" t="s">
-        <v>31</v>
-      </c>
-      <c r="C23" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
+        <v>32</v>
+      </c>
+      <c r="B24" t="s">
+        <v>32</v>
+      </c>
+      <c r="C24" t="s">
         <v>33</v>
-      </c>
-      <c r="B24" t="s">
-        <v>33</v>
-      </c>
-      <c r="C24" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
+        <v>52</v>
+      </c>
+      <c r="B25" t="s">
+        <v>34</v>
+      </c>
+      <c r="C25" t="s">
         <v>35</v>
-      </c>
-      <c r="B25" t="s">
-        <v>36</v>
-      </c>
-      <c r="C25" t="s">
-        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>